<commit_message>
Correct a super-troop row in the card tracker
Row 52 was Super Minion at Low confidence; it is Inferno Dragon, Confirmed.
Regenerated by the same openpyxl script, so only that row's cells differ.
</commit_message>
<xml_diff>
--- a/Clash_of_Cards.xlsx
+++ b/Clash_of_Cards.xlsx
@@ -3692,7 +3692,7 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Super Minion</t>
+          <t>Inferno Dragon</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
@@ -3700,14 +3700,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F53" s="15" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>coc/cards/super_troop_52_super_minion.png</t>
+          <t>coc/cards/super_troop_52_inferno_dragon.png</t>
         </is>
       </c>
     </row>

</xml_diff>